<commit_message>
Update GEO satellite anomaly risk and monthly Excel
</commit_message>
<xml_diff>
--- a/docs/data/satellite-risk/monthly/2026-09_Satellite_Anomaly_SpaceWeather.xlsx
+++ b/docs/data/satellite-risk/monthly/2026-09_Satellite_Anomaly_SpaceWeather.xlsx
@@ -14,14 +14,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Anomaly_Events!$A$3:$X$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Environment_Log!$A$2:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Environment_Log!$A$2:$I$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="137">
   <si>
     <t>SWIFT Satellite Anomaly × Space Weather — 2026-09</t>
   </si>
@@ -237,6 +237,9 @@
   </si>
   <si>
     <t>2026-09-20T11:24:59.812151Z</t>
+  </si>
+  <si>
+    <t>2026-09-20T14:29:08.384484Z</t>
   </si>
   <si>
     <t>NCEI Legacy Spacecraft Anomaly Reference</t>
@@ -1761,7 +1764,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.7109375" customWidth="1"/>
@@ -1833,8 +1836,37 @@
         <v>371.38</v>
       </c>
     </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="6">
+        <v>0.67</v>
+      </c>
+      <c r="C4" s="6">
+        <v>2.31</v>
+      </c>
+      <c r="D4" s="6">
+        <v>400.86</v>
+      </c>
+      <c r="E4" s="6">
+        <v>424.3797912597656</v>
+      </c>
+      <c r="F4" s="6">
+        <v>2.458150386810303</v>
+      </c>
+      <c r="G4" s="6">
+        <v>1.67</v>
+      </c>
+      <c r="H4" s="6">
+        <v>-10.08</v>
+      </c>
+      <c r="I4" s="6">
+        <v>369.83</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:I3"/>
+  <autoFilter ref="A2:I4"/>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
@@ -1856,7 +1888,7 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1871,39 +1903,39 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K3" s="3" t="s">
         <v>25</v>
@@ -1929,17 +1961,17 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>24</v>
@@ -1947,134 +1979,134 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -2082,10 +2114,10 @@
         <v>44</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -2093,56 +2125,56 @@
         <v>30</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="17" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="17" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="17" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="17" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="17" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="17" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>